<commit_message>
M5: deploy loss-fix guards + --explain + audit + GCP path
Root-cause fix for the first 5 paper losses (all were YES bets on
near-zero longshot buckets the market priced at 0.1-4.1c):
- engine.py: enforce min_ask_for_yes_pct (5c), min_ensemble_prob_pct
  (15%), and NBM raw-member veto (nbm_min_member_prob_pct, new lib/nbm.py).
  Each of these alone would have blocked every one of the 5 losses.
- papertrader.py: `scan --explain` per-market rule breakdown; `audit`
  command; enhanced `status`. Fixed Windows cp1252 UnicodeEncodeError
  on the explain glyphs by forcing UTF-8 stdout/stderr.
- tests/test_no_side.py: 5 NO-side unit tests (all pass).
- config.json: enable the guards.
- setup_gcp.sh: GCP e2-micro deploy path (reliable 30-min cron; GitHub
  Actions scheduled runs are throttled and fire only a few times/day).
- report.py/dashboard: 60s auto-refresh.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/papertrader/tracker.xlsx
+++ b/papertrader/tracker.xlsx
@@ -647,7 +647,7 @@
         </is>
       </c>
       <c r="T2" t="n">
-        <v>500</v>
+        <v>2000</v>
       </c>
     </row>
     <row r="3">
@@ -742,7 +742,7 @@
         </is>
       </c>
       <c r="T3" t="n">
-        <v>470</v>
+        <v>2000</v>
       </c>
     </row>
     <row r="4">

</xml_diff>